<commit_message>
fix Item Text  TEXT format
</commit_message>
<xml_diff>
--- a/invoice_automation/clients/northsky_comm/templates/Invoice_Template_no_PO.XLSX
+++ b/invoice_automation/clients/northsky_comm/templates/Invoice_Template_no_PO.XLSX
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PYTHONCODE\PDFInvoiceExtract\invoice_automation\clients\northsky_comm\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PYTHON\PDFInvoiceExtract\invoice_automation\clients\northsky_comm\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453075A5-9865-4716-A672-F1153537B1D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979DB0D8-1852-42AD-AF84-2D2E7E2C7CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9525" yWindow="1130" windowWidth="18325" windowHeight="8455" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -824,7 +824,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -849,14 +849,11 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -864,25 +861,34 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1224,7 +1230,7 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:DL6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27" style="6" customWidth="1"/>
@@ -1236,7 +1242,7 @@
     <col min="8" max="8" width="24" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30" style="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="44" style="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="44" style="8" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="20" style="6" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="23" style="6" hidden="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="40" style="7" hidden="1" bestFit="1" customWidth="1"/>
@@ -1290,14 +1296,14 @@
     <col min="69" max="69" width="15" style="6" hidden="1" bestFit="1" customWidth="1"/>
     <col min="70" max="70" width="21" style="6" hidden="1" bestFit="1" customWidth="1"/>
     <col min="71" max="71" width="33" style="6" customWidth="1"/>
-    <col min="72" max="72" width="29.5703125" style="6" customWidth="1"/>
+    <col min="72" max="72" width="29.54296875" style="6" customWidth="1"/>
     <col min="73" max="73" width="25" style="6" bestFit="1" customWidth="1"/>
     <col min="74" max="74" width="37" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="29" style="17" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="29" style="9" bestFit="1" customWidth="1"/>
     <col min="76" max="76" width="14" style="6" bestFit="1" customWidth="1"/>
     <col min="77" max="77" width="23" style="6" bestFit="1" customWidth="1"/>
     <col min="78" max="78" width="21" style="6" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="31.7109375" style="6" customWidth="1"/>
+    <col min="79" max="79" width="31.7265625" style="6" customWidth="1"/>
     <col min="80" max="80" width="20" style="6" bestFit="1" customWidth="1"/>
     <col min="81" max="81" width="19" style="6" bestFit="1" customWidth="1"/>
     <col min="82" max="82" width="18" style="6" bestFit="1" customWidth="1"/>
@@ -1336,7 +1342,7 @@
     <col min="116" max="116" width="21" style="6" hidden="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:116" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:116" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1344,1171 +1350,1277 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:116" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:116" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:116" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="K4" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="M4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="O4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="P4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="R4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="S4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="T4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="U4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="V4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="W4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="X4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AB4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AG4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AI4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AM4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AP4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AQ4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AR4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AS4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AT4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AU4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AV4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AW4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AX4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AY4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="AZ4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BA4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BB4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BC4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BD4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BE4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BF4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BG4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BH4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BI4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BJ4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BK4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BL4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BM4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BN4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BO4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BP4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BQ4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="BR4" s="11" t="s">
+      <c r="C4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="R4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="S4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="T4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="V4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="W4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="X4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AI4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AK4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AM4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AO4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AQ4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AR4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AS4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AT4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AU4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AV4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AW4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AX4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AY4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="AZ4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BA4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BB4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BC4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BD4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BE4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BF4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BG4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BH4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BI4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BJ4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BK4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BL4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BM4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BN4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BO4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BP4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BQ4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="BR4" s="10" t="s">
         <v>3</v>
       </c>
       <c r="BS4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="BT4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="BU4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="BV4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="BW4" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="BX4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="BY4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="BZ4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CA4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CB4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CC4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CD4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CE4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CF4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CG4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CH4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CI4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CJ4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CK4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CL4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CM4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CN4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CO4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CP4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CQ4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CR4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CS4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CT4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CU4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CV4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CW4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CX4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CY4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="CZ4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DA4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DB4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DC4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DD4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DE4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DF4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DG4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DH4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DI4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DJ4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DK4" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="DL4" s="10" t="s">
+      <c r="BT4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="BU4" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="BV4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="BW4" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="BX4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="BY4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="BZ4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CA4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CB4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CC4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CD4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CE4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CF4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CG4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CH4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CI4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CJ4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CK4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CL4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CM4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CN4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CO4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CP4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CQ4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CR4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CS4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CT4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CU4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CV4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CW4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CX4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CY4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="CZ4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DA4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DB4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DC4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DD4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DE4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DF4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DG4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DH4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DI4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DJ4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DK4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="DL4" s="13" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:116" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="9" t="s">
+    <row r="5" spans="1:116" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="16" t="s">
+      <c r="K5" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="L5" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="M5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="9" t="s">
+      <c r="N5" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="9" t="s">
+      <c r="O5" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="P5" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="Q5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="R5" s="9" t="s">
+      <c r="R5" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="S5" s="9" t="s">
+      <c r="S5" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T5" s="9" t="s">
+      <c r="T5" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="U5" s="9" t="s">
+      <c r="U5" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="V5" s="9" t="s">
+      <c r="V5" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="W5" s="9" t="s">
+      <c r="W5" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="X5" s="9" t="s">
+      <c r="X5" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="Y5" s="9" t="s">
+      <c r="Y5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="Z5" s="9" t="s">
+      <c r="Z5" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="AA5" s="9" t="s">
+      <c r="AA5" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="AB5" s="9" t="s">
+      <c r="AB5" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="AC5" s="9" t="s">
+      <c r="AC5" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="AD5" s="9" t="s">
+      <c r="AD5" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="AE5" s="9" t="s">
+      <c r="AE5" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="AF5" s="9" t="s">
+      <c r="AF5" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="AG5" s="9" t="s">
+      <c r="AG5" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="AH5" s="9" t="s">
+      <c r="AH5" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="AI5" s="9" t="s">
+      <c r="AI5" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="AJ5" s="9" t="s">
+      <c r="AJ5" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="AK5" s="9" t="s">
+      <c r="AK5" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="AL5" s="9" t="s">
+      <c r="AL5" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="AM5" s="9" t="s">
+      <c r="AM5" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="AN5" s="9" t="s">
+      <c r="AN5" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="AO5" s="9" t="s">
+      <c r="AO5" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="AP5" s="9" t="s">
+      <c r="AP5" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="AQ5" s="9" t="s">
+      <c r="AQ5" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="AR5" s="9" t="s">
+      <c r="AR5" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="AS5" s="9" t="s">
+      <c r="AS5" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="AT5" s="9" t="s">
+      <c r="AT5" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="AU5" s="9" t="s">
+      <c r="AU5" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="AV5" s="9" t="s">
+      <c r="AV5" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="AW5" s="9" t="s">
+      <c r="AW5" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="AX5" s="9" t="s">
+      <c r="AX5" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="AY5" s="9" t="s">
+      <c r="AY5" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="AZ5" s="9" t="s">
+      <c r="AZ5" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="BA5" s="9" t="s">
+      <c r="BA5" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="BB5" s="9" t="s">
+      <c r="BB5" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="BC5" s="9" t="s">
+      <c r="BC5" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="BD5" s="9" t="s">
+      <c r="BD5" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="BE5" s="9" t="s">
+      <c r="BE5" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="BF5" s="9" t="s">
+      <c r="BF5" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="BG5" s="9" t="s">
+      <c r="BG5" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="BH5" s="9" t="s">
+      <c r="BH5" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="BI5" s="9" t="s">
+      <c r="BI5" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="BJ5" s="9" t="s">
+      <c r="BJ5" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="BK5" s="9" t="s">
+      <c r="BK5" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="BL5" s="9" t="s">
+      <c r="BL5" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="BM5" s="9" t="s">
+      <c r="BM5" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="BN5" s="9" t="s">
+      <c r="BN5" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="BO5" s="9" t="s">
+      <c r="BO5" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="BP5" s="9" t="s">
+      <c r="BP5" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="BQ5" s="9" t="s">
+      <c r="BQ5" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="BR5" s="9" t="s">
+      <c r="BR5" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="BS5" s="8" t="s">
+      <c r="BS5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="BT5" s="8" t="s">
+      <c r="BT5" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="BU5" s="8" t="s">
+      <c r="BU5" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="BV5" s="8" t="s">
+      <c r="BV5" s="18" t="s">
         <v>77</v>
       </c>
       <c r="BW5" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="BX5" s="8" t="s">
+      <c r="BX5" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="BY5" s="8" t="s">
+      <c r="BY5" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="BZ5" s="8" t="s">
+      <c r="BZ5" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="CA5" s="8" t="s">
+      <c r="CA5" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="CB5" s="8" t="s">
+      <c r="CB5" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="CC5" s="8" t="s">
+      <c r="CC5" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="CD5" s="8" t="s">
+      <c r="CD5" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="CE5" s="8" t="s">
+      <c r="CE5" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="CF5" s="8" t="s">
+      <c r="CF5" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="CG5" s="8" t="s">
+      <c r="CG5" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="CH5" s="8" t="s">
+      <c r="CH5" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="CI5" s="8" t="s">
+      <c r="CI5" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="CJ5" s="8" t="s">
+      <c r="CJ5" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="CK5" s="8" t="s">
+      <c r="CK5" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="CL5" s="8" t="s">
+      <c r="CL5" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="CM5" s="8" t="s">
+      <c r="CM5" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="CN5" s="8" t="s">
+      <c r="CN5" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="CO5" s="8" t="s">
+      <c r="CO5" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="CP5" s="8" t="s">
+      <c r="CP5" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="CQ5" s="8" t="s">
+      <c r="CQ5" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="CR5" s="8" t="s">
+      <c r="CR5" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="CS5" s="8" t="s">
+      <c r="CS5" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="CT5" s="8" t="s">
+      <c r="CT5" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="CU5" s="8" t="s">
+      <c r="CU5" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="CV5" s="8" t="s">
+      <c r="CV5" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="CW5" s="8" t="s">
+      <c r="CW5" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="CX5" s="8" t="s">
+      <c r="CX5" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="CY5" s="8" t="s">
+      <c r="CY5" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="CZ5" s="8" t="s">
+      <c r="CZ5" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="DA5" s="8" t="s">
+      <c r="DA5" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="DB5" s="8" t="s">
+      <c r="DB5" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="DC5" s="8" t="s">
+      <c r="DC5" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="DD5" s="8" t="s">
+      <c r="DD5" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="DE5" s="8" t="s">
+      <c r="DE5" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="DF5" s="8" t="s">
+      <c r="DF5" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="DG5" s="8" t="s">
+      <c r="DG5" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="DH5" s="8" t="s">
+      <c r="DH5" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="DI5" s="8" t="s">
+      <c r="DI5" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="DJ5" s="8" t="s">
+      <c r="DJ5" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="DK5" s="8" t="s">
+      <c r="DK5" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="DL5" s="8" t="s">
+      <c r="DL5" s="18" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="1:116" s="5" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:116" s="5" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="J6" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="K6" s="16" t="s">
+      <c r="K6" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="L6" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="M6" s="9" t="s">
+      <c r="M6" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="N6" s="9" t="s">
+      <c r="N6" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="O6" s="9" t="s">
+      <c r="O6" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="P6" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="Q6" s="9" t="s">
+      <c r="Q6" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="R6" s="9" t="s">
+      <c r="R6" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="S6" s="9" t="s">
+      <c r="S6" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="T6" s="9" t="s">
+      <c r="T6" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="U6" s="9" t="s">
+      <c r="U6" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="V6" s="9" t="s">
+      <c r="V6" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="W6" s="9" t="s">
+      <c r="W6" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="X6" s="9" t="s">
+      <c r="X6" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="Y6" s="9" t="s">
+      <c r="Y6" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="Z6" s="9" t="s">
+      <c r="Z6" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="AA6" s="9" t="s">
+      <c r="AA6" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="AB6" s="9" t="s">
+      <c r="AB6" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="AC6" s="9" t="s">
+      <c r="AC6" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="AD6" s="9" t="s">
+      <c r="AD6" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="AE6" s="9" t="s">
+      <c r="AE6" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="AF6" s="9" t="s">
+      <c r="AF6" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="AG6" s="9" t="s">
+      <c r="AG6" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="AH6" s="9" t="s">
+      <c r="AH6" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="AI6" s="9" t="s">
+      <c r="AI6" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="AJ6" s="9" t="s">
+      <c r="AJ6" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="AK6" s="9" t="s">
+      <c r="AK6" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="AL6" s="9" t="s">
+      <c r="AL6" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="AM6" s="9" t="s">
+      <c r="AM6" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="AN6" s="9" t="s">
+      <c r="AN6" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="AO6" s="9" t="s">
+      <c r="AO6" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="AP6" s="9" t="s">
+      <c r="AP6" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="AQ6" s="9" t="s">
+      <c r="AQ6" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="AR6" s="9" t="s">
+      <c r="AR6" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="AS6" s="9" t="s">
+      <c r="AS6" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="AT6" s="9" t="s">
+      <c r="AT6" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="AU6" s="9" t="s">
+      <c r="AU6" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="AV6" s="9" t="s">
+      <c r="AV6" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="AW6" s="9" t="s">
+      <c r="AW6" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="AX6" s="9" t="s">
+      <c r="AX6" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="AY6" s="9" t="s">
+      <c r="AY6" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="AZ6" s="9" t="s">
+      <c r="AZ6" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="BA6" s="9" t="s">
+      <c r="BA6" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="BB6" s="9" t="s">
+      <c r="BB6" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="BC6" s="9" t="s">
+      <c r="BC6" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="BD6" s="9" t="s">
+      <c r="BD6" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="BE6" s="9" t="s">
+      <c r="BE6" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="BF6" s="9" t="s">
+      <c r="BF6" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="BG6" s="9" t="s">
+      <c r="BG6" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="BH6" s="9" t="s">
+      <c r="BH6" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="BI6" s="9" t="s">
+      <c r="BI6" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="BJ6" s="9" t="s">
+      <c r="BJ6" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="BK6" s="9" t="s">
+      <c r="BK6" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="BL6" s="9" t="s">
+      <c r="BL6" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="BM6" s="9" t="s">
+      <c r="BM6" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="BN6" s="9" t="s">
+      <c r="BN6" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="BO6" s="9" t="s">
+      <c r="BO6" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="BP6" s="9" t="s">
+      <c r="BP6" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="BQ6" s="9" t="s">
+      <c r="BQ6" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="BR6" s="9" t="s">
+      <c r="BR6" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="BS6" s="8" t="s">
+      <c r="BS6" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="BT6" s="8" t="s">
+      <c r="BT6" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="BU6" s="8" t="s">
+      <c r="BU6" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="BV6" s="8" t="s">
+      <c r="BV6" s="18" t="s">
         <v>191</v>
       </c>
       <c r="BW6" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="BX6" s="8" t="s">
+      <c r="BX6" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="BY6" s="8" t="s">
+      <c r="BY6" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="BZ6" s="8" t="s">
+      <c r="BZ6" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="CA6" s="8" t="s">
+      <c r="CA6" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="CB6" s="8" t="s">
+      <c r="CB6" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="CC6" s="8" t="s">
+      <c r="CC6" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="CD6" s="8" t="s">
+      <c r="CD6" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="CE6" s="8" t="s">
+      <c r="CE6" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="CF6" s="8" t="s">
+      <c r="CF6" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="CG6" s="8" t="s">
+      <c r="CG6" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="CH6" s="8" t="s">
+      <c r="CH6" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="CI6" s="8" t="s">
+      <c r="CI6" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="CJ6" s="8" t="s">
+      <c r="CJ6" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="CK6" s="8" t="s">
+      <c r="CK6" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="CL6" s="8" t="s">
+      <c r="CL6" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="CM6" s="8" t="s">
+      <c r="CM6" s="18" t="s">
         <v>208</v>
       </c>
-      <c r="CN6" s="8" t="s">
+      <c r="CN6" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="CO6" s="8" t="s">
+      <c r="CO6" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="CP6" s="8" t="s">
+      <c r="CP6" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="CQ6" s="8" t="s">
+      <c r="CQ6" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="CR6" s="8" t="s">
+      <c r="CR6" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="CS6" s="8" t="s">
+      <c r="CS6" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="CT6" s="8" t="s">
+      <c r="CT6" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="CU6" s="8" t="s">
+      <c r="CU6" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="CV6" s="8" t="s">
+      <c r="CV6" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="CW6" s="8" t="s">
+      <c r="CW6" s="18" t="s">
         <v>218</v>
       </c>
-      <c r="CX6" s="8" t="s">
+      <c r="CX6" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="CY6" s="8" t="s">
+      <c r="CY6" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="CZ6" s="8" t="s">
+      <c r="CZ6" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="DA6" s="8" t="s">
+      <c r="DA6" s="18" t="s">
         <v>222</v>
       </c>
-      <c r="DB6" s="8" t="s">
+      <c r="DB6" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="DC6" s="8" t="s">
+      <c r="DC6" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="DD6" s="8" t="s">
+      <c r="DD6" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="DE6" s="8" t="s">
+      <c r="DE6" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="DF6" s="8" t="s">
+      <c r="DF6" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="DG6" s="8" t="s">
+      <c r="DG6" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="DH6" s="8" t="s">
+      <c r="DH6" s="18" t="s">
         <v>229</v>
       </c>
-      <c r="DI6" s="8" t="s">
+      <c r="DI6" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="DJ6" s="8" t="s">
+      <c r="DJ6" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="DK6" s="8" t="s">
+      <c r="DK6" s="18" t="s">
         <v>232</v>
       </c>
-      <c r="DL6" s="8" t="s">
+      <c r="DL6" s="18" t="s">
         <v>233</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="346">
-    <mergeCell ref="B4"/>
-    <mergeCell ref="C4"/>
-    <mergeCell ref="D4"/>
-    <mergeCell ref="E4"/>
-    <mergeCell ref="F4"/>
-    <mergeCell ref="G4"/>
-    <mergeCell ref="H4"/>
-    <mergeCell ref="I4"/>
-    <mergeCell ref="J4"/>
-    <mergeCell ref="K4"/>
-    <mergeCell ref="L4"/>
-    <mergeCell ref="M4"/>
-    <mergeCell ref="N4"/>
-    <mergeCell ref="O4"/>
-    <mergeCell ref="P4"/>
-    <mergeCell ref="Q4"/>
-    <mergeCell ref="R4"/>
-    <mergeCell ref="S4"/>
-    <mergeCell ref="T4"/>
-    <mergeCell ref="U4"/>
-    <mergeCell ref="V4"/>
-    <mergeCell ref="W4"/>
-    <mergeCell ref="X4"/>
-    <mergeCell ref="Y4"/>
-    <mergeCell ref="Z4"/>
-    <mergeCell ref="AA4"/>
-    <mergeCell ref="AB4"/>
-    <mergeCell ref="AC4"/>
-    <mergeCell ref="AD4"/>
-    <mergeCell ref="AE4"/>
-    <mergeCell ref="AF4"/>
-    <mergeCell ref="AG4"/>
-    <mergeCell ref="AH4"/>
-    <mergeCell ref="AI4"/>
-    <mergeCell ref="AJ4"/>
-    <mergeCell ref="AK4"/>
-    <mergeCell ref="AL4"/>
-    <mergeCell ref="AM4"/>
-    <mergeCell ref="AN4"/>
-    <mergeCell ref="AO4"/>
-    <mergeCell ref="AP4"/>
-    <mergeCell ref="AQ4"/>
-    <mergeCell ref="AR4"/>
-    <mergeCell ref="AS4"/>
-    <mergeCell ref="AT4"/>
-    <mergeCell ref="AU4"/>
-    <mergeCell ref="AV4"/>
-    <mergeCell ref="AW4"/>
-    <mergeCell ref="AX4"/>
-    <mergeCell ref="AY4"/>
-    <mergeCell ref="AZ4"/>
-    <mergeCell ref="BA4"/>
-    <mergeCell ref="BB4"/>
-    <mergeCell ref="BC4"/>
-    <mergeCell ref="BD4"/>
-    <mergeCell ref="BE4"/>
-    <mergeCell ref="BF4"/>
-    <mergeCell ref="BG4"/>
-    <mergeCell ref="BH4"/>
-    <mergeCell ref="BI4"/>
-    <mergeCell ref="BJ4"/>
-    <mergeCell ref="BK4"/>
-    <mergeCell ref="BL4"/>
-    <mergeCell ref="BM4"/>
-    <mergeCell ref="BN4"/>
-    <mergeCell ref="BO4"/>
-    <mergeCell ref="BP4"/>
-    <mergeCell ref="BQ4"/>
-    <mergeCell ref="BR4"/>
-    <mergeCell ref="BT4"/>
-    <mergeCell ref="BU4"/>
-    <mergeCell ref="BV4"/>
-    <mergeCell ref="BW4"/>
-    <mergeCell ref="BX4"/>
-    <mergeCell ref="BY4"/>
-    <mergeCell ref="BZ4"/>
-    <mergeCell ref="CA4"/>
-    <mergeCell ref="CB4"/>
-    <mergeCell ref="CC4"/>
-    <mergeCell ref="CD4"/>
-    <mergeCell ref="CE4"/>
-    <mergeCell ref="CF4"/>
-    <mergeCell ref="CG4"/>
-    <mergeCell ref="CH4"/>
-    <mergeCell ref="CI4"/>
-    <mergeCell ref="CJ4"/>
-    <mergeCell ref="CK4"/>
-    <mergeCell ref="CL4"/>
-    <mergeCell ref="CM4"/>
-    <mergeCell ref="CN4"/>
-    <mergeCell ref="CO4"/>
-    <mergeCell ref="CP4"/>
-    <mergeCell ref="CQ4"/>
-    <mergeCell ref="CR4"/>
-    <mergeCell ref="CS4"/>
-    <mergeCell ref="CT4"/>
-    <mergeCell ref="CU4"/>
-    <mergeCell ref="CV4"/>
-    <mergeCell ref="CW4"/>
-    <mergeCell ref="CX4"/>
-    <mergeCell ref="CY4"/>
-    <mergeCell ref="CZ4"/>
-    <mergeCell ref="DA4"/>
-    <mergeCell ref="DB4"/>
-    <mergeCell ref="DC4"/>
-    <mergeCell ref="DD4"/>
-    <mergeCell ref="DE4"/>
-    <mergeCell ref="DF4"/>
+    <mergeCell ref="DL6"/>
+    <mergeCell ref="DC6"/>
+    <mergeCell ref="DD6"/>
+    <mergeCell ref="DE6"/>
+    <mergeCell ref="DF6"/>
+    <mergeCell ref="DG6"/>
+    <mergeCell ref="DH6"/>
+    <mergeCell ref="DI6"/>
+    <mergeCell ref="DJ6"/>
+    <mergeCell ref="DK6"/>
+    <mergeCell ref="CT6"/>
+    <mergeCell ref="CU6"/>
+    <mergeCell ref="CV6"/>
+    <mergeCell ref="CW6"/>
+    <mergeCell ref="CX6"/>
+    <mergeCell ref="CY6"/>
+    <mergeCell ref="CZ6"/>
+    <mergeCell ref="DA6"/>
+    <mergeCell ref="DB6"/>
+    <mergeCell ref="CK6"/>
+    <mergeCell ref="CL6"/>
+    <mergeCell ref="CM6"/>
+    <mergeCell ref="CN6"/>
+    <mergeCell ref="CO6"/>
+    <mergeCell ref="CP6"/>
+    <mergeCell ref="CQ6"/>
+    <mergeCell ref="CR6"/>
+    <mergeCell ref="CS6"/>
+    <mergeCell ref="CB6"/>
+    <mergeCell ref="CC6"/>
+    <mergeCell ref="CD6"/>
+    <mergeCell ref="CE6"/>
+    <mergeCell ref="CF6"/>
+    <mergeCell ref="CG6"/>
+    <mergeCell ref="CH6"/>
+    <mergeCell ref="CI6"/>
+    <mergeCell ref="CJ6"/>
+    <mergeCell ref="BS6"/>
+    <mergeCell ref="BT6"/>
+    <mergeCell ref="BU6"/>
+    <mergeCell ref="BV6"/>
+    <mergeCell ref="BW6"/>
+    <mergeCell ref="BX6"/>
+    <mergeCell ref="BY6"/>
+    <mergeCell ref="BZ6"/>
+    <mergeCell ref="CA6"/>
+    <mergeCell ref="BJ6"/>
+    <mergeCell ref="BK6"/>
+    <mergeCell ref="BL6"/>
+    <mergeCell ref="BM6"/>
+    <mergeCell ref="BN6"/>
+    <mergeCell ref="BO6"/>
+    <mergeCell ref="BP6"/>
+    <mergeCell ref="BQ6"/>
+    <mergeCell ref="BR6"/>
+    <mergeCell ref="BA6"/>
+    <mergeCell ref="BB6"/>
+    <mergeCell ref="BC6"/>
+    <mergeCell ref="BD6"/>
+    <mergeCell ref="BE6"/>
+    <mergeCell ref="BF6"/>
+    <mergeCell ref="BG6"/>
+    <mergeCell ref="BH6"/>
+    <mergeCell ref="BI6"/>
+    <mergeCell ref="AR6"/>
+    <mergeCell ref="AS6"/>
+    <mergeCell ref="AT6"/>
+    <mergeCell ref="AU6"/>
+    <mergeCell ref="AV6"/>
+    <mergeCell ref="AW6"/>
+    <mergeCell ref="AX6"/>
+    <mergeCell ref="AY6"/>
+    <mergeCell ref="AZ6"/>
+    <mergeCell ref="AI6"/>
+    <mergeCell ref="AJ6"/>
+    <mergeCell ref="AK6"/>
+    <mergeCell ref="AL6"/>
+    <mergeCell ref="AM6"/>
+    <mergeCell ref="AN6"/>
+    <mergeCell ref="AO6"/>
+    <mergeCell ref="AP6"/>
+    <mergeCell ref="AQ6"/>
+    <mergeCell ref="Z6"/>
+    <mergeCell ref="AA6"/>
+    <mergeCell ref="AB6"/>
+    <mergeCell ref="AC6"/>
+    <mergeCell ref="AD6"/>
+    <mergeCell ref="AE6"/>
+    <mergeCell ref="AF6"/>
+    <mergeCell ref="AG6"/>
+    <mergeCell ref="AH6"/>
+    <mergeCell ref="Q6"/>
+    <mergeCell ref="R6"/>
+    <mergeCell ref="S6"/>
+    <mergeCell ref="T6"/>
+    <mergeCell ref="U6"/>
+    <mergeCell ref="V6"/>
+    <mergeCell ref="W6"/>
+    <mergeCell ref="X6"/>
+    <mergeCell ref="Y6"/>
+    <mergeCell ref="DE5"/>
+    <mergeCell ref="DF5"/>
+    <mergeCell ref="DG5"/>
+    <mergeCell ref="DH5"/>
+    <mergeCell ref="DI5"/>
+    <mergeCell ref="DJ5"/>
+    <mergeCell ref="DK5"/>
+    <mergeCell ref="DL5"/>
+    <mergeCell ref="A6"/>
+    <mergeCell ref="B6"/>
+    <mergeCell ref="C6"/>
+    <mergeCell ref="D6"/>
+    <mergeCell ref="E6"/>
+    <mergeCell ref="F6"/>
+    <mergeCell ref="G6"/>
+    <mergeCell ref="H6"/>
+    <mergeCell ref="I6"/>
+    <mergeCell ref="J6"/>
+    <mergeCell ref="K6"/>
+    <mergeCell ref="L6"/>
+    <mergeCell ref="M6"/>
+    <mergeCell ref="N6"/>
+    <mergeCell ref="O6"/>
+    <mergeCell ref="P6"/>
+    <mergeCell ref="CV5"/>
+    <mergeCell ref="CW5"/>
+    <mergeCell ref="CX5"/>
+    <mergeCell ref="CY5"/>
+    <mergeCell ref="CZ5"/>
+    <mergeCell ref="DA5"/>
+    <mergeCell ref="DB5"/>
+    <mergeCell ref="DC5"/>
+    <mergeCell ref="DD5"/>
+    <mergeCell ref="CM5"/>
+    <mergeCell ref="CN5"/>
+    <mergeCell ref="CO5"/>
+    <mergeCell ref="CP5"/>
+    <mergeCell ref="CQ5"/>
+    <mergeCell ref="CR5"/>
+    <mergeCell ref="CS5"/>
+    <mergeCell ref="CT5"/>
+    <mergeCell ref="CU5"/>
+    <mergeCell ref="CD5"/>
+    <mergeCell ref="CE5"/>
+    <mergeCell ref="CF5"/>
+    <mergeCell ref="CG5"/>
+    <mergeCell ref="CH5"/>
+    <mergeCell ref="CI5"/>
+    <mergeCell ref="CJ5"/>
+    <mergeCell ref="CK5"/>
+    <mergeCell ref="CL5"/>
+    <mergeCell ref="BU5"/>
+    <mergeCell ref="BV5"/>
+    <mergeCell ref="BW5"/>
+    <mergeCell ref="BX5"/>
+    <mergeCell ref="BY5"/>
+    <mergeCell ref="BZ5"/>
+    <mergeCell ref="CA5"/>
+    <mergeCell ref="CB5"/>
+    <mergeCell ref="CC5"/>
+    <mergeCell ref="BL5"/>
+    <mergeCell ref="BM5"/>
+    <mergeCell ref="BN5"/>
+    <mergeCell ref="BO5"/>
+    <mergeCell ref="BP5"/>
+    <mergeCell ref="BQ5"/>
+    <mergeCell ref="BR5"/>
+    <mergeCell ref="BS5"/>
+    <mergeCell ref="BT5"/>
+    <mergeCell ref="BC5"/>
+    <mergeCell ref="BD5"/>
+    <mergeCell ref="BE5"/>
+    <mergeCell ref="BF5"/>
+    <mergeCell ref="BG5"/>
+    <mergeCell ref="BH5"/>
+    <mergeCell ref="BI5"/>
+    <mergeCell ref="BJ5"/>
+    <mergeCell ref="BK5"/>
+    <mergeCell ref="AT5"/>
+    <mergeCell ref="AU5"/>
+    <mergeCell ref="AV5"/>
+    <mergeCell ref="AW5"/>
+    <mergeCell ref="AX5"/>
+    <mergeCell ref="AY5"/>
+    <mergeCell ref="AZ5"/>
+    <mergeCell ref="BA5"/>
+    <mergeCell ref="BB5"/>
+    <mergeCell ref="AK5"/>
+    <mergeCell ref="AL5"/>
+    <mergeCell ref="AM5"/>
+    <mergeCell ref="AN5"/>
+    <mergeCell ref="AO5"/>
+    <mergeCell ref="AP5"/>
+    <mergeCell ref="AQ5"/>
+    <mergeCell ref="AR5"/>
+    <mergeCell ref="AS5"/>
+    <mergeCell ref="AB5"/>
+    <mergeCell ref="AC5"/>
+    <mergeCell ref="AD5"/>
+    <mergeCell ref="AE5"/>
+    <mergeCell ref="AF5"/>
+    <mergeCell ref="AG5"/>
+    <mergeCell ref="AH5"/>
+    <mergeCell ref="AI5"/>
+    <mergeCell ref="AJ5"/>
+    <mergeCell ref="S5"/>
+    <mergeCell ref="T5"/>
+    <mergeCell ref="U5"/>
+    <mergeCell ref="V5"/>
+    <mergeCell ref="W5"/>
+    <mergeCell ref="X5"/>
+    <mergeCell ref="Y5"/>
+    <mergeCell ref="Z5"/>
+    <mergeCell ref="AA5"/>
     <mergeCell ref="DG4"/>
     <mergeCell ref="DH4"/>
     <mergeCell ref="DI4"/>
@@ -2533,220 +2645,114 @@
     <mergeCell ref="P5"/>
     <mergeCell ref="Q5"/>
     <mergeCell ref="R5"/>
-    <mergeCell ref="S5"/>
-    <mergeCell ref="T5"/>
-    <mergeCell ref="U5"/>
-    <mergeCell ref="V5"/>
-    <mergeCell ref="W5"/>
-    <mergeCell ref="X5"/>
-    <mergeCell ref="Y5"/>
-    <mergeCell ref="Z5"/>
-    <mergeCell ref="AA5"/>
-    <mergeCell ref="AB5"/>
-    <mergeCell ref="AC5"/>
-    <mergeCell ref="AD5"/>
-    <mergeCell ref="AE5"/>
-    <mergeCell ref="AF5"/>
-    <mergeCell ref="AG5"/>
-    <mergeCell ref="AH5"/>
-    <mergeCell ref="AI5"/>
-    <mergeCell ref="AJ5"/>
-    <mergeCell ref="AK5"/>
-    <mergeCell ref="AL5"/>
-    <mergeCell ref="AM5"/>
-    <mergeCell ref="AN5"/>
-    <mergeCell ref="AO5"/>
-    <mergeCell ref="AP5"/>
-    <mergeCell ref="AQ5"/>
-    <mergeCell ref="AR5"/>
-    <mergeCell ref="AS5"/>
-    <mergeCell ref="AT5"/>
-    <mergeCell ref="AU5"/>
-    <mergeCell ref="AV5"/>
-    <mergeCell ref="AW5"/>
-    <mergeCell ref="AX5"/>
-    <mergeCell ref="AY5"/>
-    <mergeCell ref="AZ5"/>
-    <mergeCell ref="BA5"/>
-    <mergeCell ref="BB5"/>
-    <mergeCell ref="BC5"/>
-    <mergeCell ref="BD5"/>
-    <mergeCell ref="BE5"/>
-    <mergeCell ref="BF5"/>
-    <mergeCell ref="BG5"/>
-    <mergeCell ref="BH5"/>
-    <mergeCell ref="BI5"/>
-    <mergeCell ref="BJ5"/>
-    <mergeCell ref="BK5"/>
-    <mergeCell ref="BL5"/>
-    <mergeCell ref="BM5"/>
-    <mergeCell ref="BN5"/>
-    <mergeCell ref="BO5"/>
-    <mergeCell ref="BP5"/>
-    <mergeCell ref="BQ5"/>
-    <mergeCell ref="BR5"/>
-    <mergeCell ref="BS5"/>
-    <mergeCell ref="BT5"/>
-    <mergeCell ref="BU5"/>
-    <mergeCell ref="BV5"/>
-    <mergeCell ref="BW5"/>
-    <mergeCell ref="BX5"/>
-    <mergeCell ref="BY5"/>
-    <mergeCell ref="BZ5"/>
-    <mergeCell ref="CA5"/>
-    <mergeCell ref="CB5"/>
-    <mergeCell ref="CC5"/>
-    <mergeCell ref="CD5"/>
-    <mergeCell ref="CE5"/>
-    <mergeCell ref="CF5"/>
-    <mergeCell ref="CG5"/>
-    <mergeCell ref="CH5"/>
-    <mergeCell ref="CI5"/>
-    <mergeCell ref="CJ5"/>
-    <mergeCell ref="CK5"/>
-    <mergeCell ref="CL5"/>
-    <mergeCell ref="CM5"/>
-    <mergeCell ref="CN5"/>
-    <mergeCell ref="CO5"/>
-    <mergeCell ref="CP5"/>
-    <mergeCell ref="CQ5"/>
-    <mergeCell ref="CR5"/>
-    <mergeCell ref="CS5"/>
-    <mergeCell ref="CT5"/>
-    <mergeCell ref="CU5"/>
-    <mergeCell ref="CV5"/>
-    <mergeCell ref="CW5"/>
-    <mergeCell ref="CX5"/>
-    <mergeCell ref="CY5"/>
-    <mergeCell ref="CZ5"/>
-    <mergeCell ref="DA5"/>
-    <mergeCell ref="DB5"/>
-    <mergeCell ref="DC5"/>
-    <mergeCell ref="DD5"/>
-    <mergeCell ref="DE5"/>
-    <mergeCell ref="DF5"/>
-    <mergeCell ref="DG5"/>
-    <mergeCell ref="DH5"/>
-    <mergeCell ref="DI5"/>
-    <mergeCell ref="DJ5"/>
-    <mergeCell ref="DK5"/>
-    <mergeCell ref="DL5"/>
-    <mergeCell ref="A6"/>
-    <mergeCell ref="B6"/>
-    <mergeCell ref="C6"/>
-    <mergeCell ref="D6"/>
-    <mergeCell ref="E6"/>
-    <mergeCell ref="F6"/>
-    <mergeCell ref="G6"/>
-    <mergeCell ref="H6"/>
-    <mergeCell ref="I6"/>
-    <mergeCell ref="J6"/>
-    <mergeCell ref="K6"/>
-    <mergeCell ref="L6"/>
-    <mergeCell ref="M6"/>
-    <mergeCell ref="N6"/>
-    <mergeCell ref="O6"/>
-    <mergeCell ref="P6"/>
-    <mergeCell ref="Q6"/>
-    <mergeCell ref="R6"/>
-    <mergeCell ref="S6"/>
-    <mergeCell ref="T6"/>
-    <mergeCell ref="U6"/>
-    <mergeCell ref="V6"/>
-    <mergeCell ref="W6"/>
-    <mergeCell ref="X6"/>
-    <mergeCell ref="Y6"/>
-    <mergeCell ref="Z6"/>
-    <mergeCell ref="AA6"/>
-    <mergeCell ref="AB6"/>
-    <mergeCell ref="AC6"/>
-    <mergeCell ref="AD6"/>
-    <mergeCell ref="AE6"/>
-    <mergeCell ref="AF6"/>
-    <mergeCell ref="AG6"/>
-    <mergeCell ref="AH6"/>
-    <mergeCell ref="AI6"/>
-    <mergeCell ref="AJ6"/>
-    <mergeCell ref="AK6"/>
-    <mergeCell ref="AL6"/>
-    <mergeCell ref="AM6"/>
-    <mergeCell ref="AN6"/>
-    <mergeCell ref="AO6"/>
-    <mergeCell ref="AP6"/>
-    <mergeCell ref="AQ6"/>
-    <mergeCell ref="AR6"/>
-    <mergeCell ref="AS6"/>
-    <mergeCell ref="AT6"/>
-    <mergeCell ref="AU6"/>
-    <mergeCell ref="AV6"/>
-    <mergeCell ref="AW6"/>
-    <mergeCell ref="AX6"/>
-    <mergeCell ref="AY6"/>
-    <mergeCell ref="AZ6"/>
-    <mergeCell ref="BA6"/>
-    <mergeCell ref="BB6"/>
-    <mergeCell ref="BC6"/>
-    <mergeCell ref="BD6"/>
-    <mergeCell ref="BE6"/>
-    <mergeCell ref="BF6"/>
-    <mergeCell ref="BG6"/>
-    <mergeCell ref="BH6"/>
-    <mergeCell ref="BI6"/>
-    <mergeCell ref="BJ6"/>
-    <mergeCell ref="BK6"/>
-    <mergeCell ref="BL6"/>
-    <mergeCell ref="BM6"/>
-    <mergeCell ref="BN6"/>
-    <mergeCell ref="BO6"/>
-    <mergeCell ref="BP6"/>
-    <mergeCell ref="BQ6"/>
-    <mergeCell ref="BR6"/>
-    <mergeCell ref="BS6"/>
-    <mergeCell ref="BT6"/>
-    <mergeCell ref="BU6"/>
-    <mergeCell ref="BV6"/>
-    <mergeCell ref="BW6"/>
-    <mergeCell ref="BX6"/>
-    <mergeCell ref="BY6"/>
-    <mergeCell ref="BZ6"/>
-    <mergeCell ref="CA6"/>
-    <mergeCell ref="CB6"/>
-    <mergeCell ref="CC6"/>
-    <mergeCell ref="CD6"/>
-    <mergeCell ref="CE6"/>
-    <mergeCell ref="CF6"/>
-    <mergeCell ref="CG6"/>
-    <mergeCell ref="CH6"/>
-    <mergeCell ref="CI6"/>
-    <mergeCell ref="CJ6"/>
-    <mergeCell ref="CK6"/>
-    <mergeCell ref="CL6"/>
-    <mergeCell ref="CM6"/>
-    <mergeCell ref="CN6"/>
-    <mergeCell ref="CO6"/>
-    <mergeCell ref="CP6"/>
-    <mergeCell ref="CQ6"/>
-    <mergeCell ref="CR6"/>
-    <mergeCell ref="CS6"/>
-    <mergeCell ref="CT6"/>
-    <mergeCell ref="CU6"/>
-    <mergeCell ref="CV6"/>
-    <mergeCell ref="CW6"/>
-    <mergeCell ref="CX6"/>
-    <mergeCell ref="CY6"/>
-    <mergeCell ref="CZ6"/>
-    <mergeCell ref="DA6"/>
-    <mergeCell ref="DB6"/>
-    <mergeCell ref="DL6"/>
-    <mergeCell ref="DC6"/>
-    <mergeCell ref="DD6"/>
-    <mergeCell ref="DE6"/>
-    <mergeCell ref="DF6"/>
-    <mergeCell ref="DG6"/>
-    <mergeCell ref="DH6"/>
-    <mergeCell ref="DI6"/>
-    <mergeCell ref="DJ6"/>
-    <mergeCell ref="DK6"/>
+    <mergeCell ref="CX4"/>
+    <mergeCell ref="CY4"/>
+    <mergeCell ref="CZ4"/>
+    <mergeCell ref="DA4"/>
+    <mergeCell ref="DB4"/>
+    <mergeCell ref="DC4"/>
+    <mergeCell ref="DD4"/>
+    <mergeCell ref="DE4"/>
+    <mergeCell ref="DF4"/>
+    <mergeCell ref="CO4"/>
+    <mergeCell ref="CP4"/>
+    <mergeCell ref="CQ4"/>
+    <mergeCell ref="CR4"/>
+    <mergeCell ref="CS4"/>
+    <mergeCell ref="CT4"/>
+    <mergeCell ref="CU4"/>
+    <mergeCell ref="CV4"/>
+    <mergeCell ref="CW4"/>
+    <mergeCell ref="CF4"/>
+    <mergeCell ref="CG4"/>
+    <mergeCell ref="CH4"/>
+    <mergeCell ref="CI4"/>
+    <mergeCell ref="CJ4"/>
+    <mergeCell ref="CK4"/>
+    <mergeCell ref="CL4"/>
+    <mergeCell ref="CM4"/>
+    <mergeCell ref="CN4"/>
+    <mergeCell ref="BW4"/>
+    <mergeCell ref="BX4"/>
+    <mergeCell ref="BY4"/>
+    <mergeCell ref="BZ4"/>
+    <mergeCell ref="CA4"/>
+    <mergeCell ref="CB4"/>
+    <mergeCell ref="CC4"/>
+    <mergeCell ref="CD4"/>
+    <mergeCell ref="CE4"/>
+    <mergeCell ref="BM4"/>
+    <mergeCell ref="BN4"/>
+    <mergeCell ref="BO4"/>
+    <mergeCell ref="BP4"/>
+    <mergeCell ref="BQ4"/>
+    <mergeCell ref="BR4"/>
+    <mergeCell ref="BT4"/>
+    <mergeCell ref="BU4"/>
+    <mergeCell ref="BV4"/>
+    <mergeCell ref="BD4"/>
+    <mergeCell ref="BE4"/>
+    <mergeCell ref="BF4"/>
+    <mergeCell ref="BG4"/>
+    <mergeCell ref="BH4"/>
+    <mergeCell ref="BI4"/>
+    <mergeCell ref="BJ4"/>
+    <mergeCell ref="BK4"/>
+    <mergeCell ref="BL4"/>
+    <mergeCell ref="AU4"/>
+    <mergeCell ref="AV4"/>
+    <mergeCell ref="AW4"/>
+    <mergeCell ref="AX4"/>
+    <mergeCell ref="AY4"/>
+    <mergeCell ref="AZ4"/>
+    <mergeCell ref="BA4"/>
+    <mergeCell ref="BB4"/>
+    <mergeCell ref="BC4"/>
+    <mergeCell ref="AL4"/>
+    <mergeCell ref="AM4"/>
+    <mergeCell ref="AN4"/>
+    <mergeCell ref="AO4"/>
+    <mergeCell ref="AP4"/>
+    <mergeCell ref="AQ4"/>
+    <mergeCell ref="AR4"/>
+    <mergeCell ref="AS4"/>
+    <mergeCell ref="AT4"/>
+    <mergeCell ref="AC4"/>
+    <mergeCell ref="AD4"/>
+    <mergeCell ref="AE4"/>
+    <mergeCell ref="AF4"/>
+    <mergeCell ref="AG4"/>
+    <mergeCell ref="AH4"/>
+    <mergeCell ref="AI4"/>
+    <mergeCell ref="AJ4"/>
+    <mergeCell ref="AK4"/>
+    <mergeCell ref="T4"/>
+    <mergeCell ref="U4"/>
+    <mergeCell ref="V4"/>
+    <mergeCell ref="W4"/>
+    <mergeCell ref="X4"/>
+    <mergeCell ref="Y4"/>
+    <mergeCell ref="Z4"/>
+    <mergeCell ref="AA4"/>
+    <mergeCell ref="AB4"/>
+    <mergeCell ref="K4"/>
+    <mergeCell ref="L4"/>
+    <mergeCell ref="M4"/>
+    <mergeCell ref="N4"/>
+    <mergeCell ref="O4"/>
+    <mergeCell ref="P4"/>
+    <mergeCell ref="Q4"/>
+    <mergeCell ref="R4"/>
+    <mergeCell ref="S4"/>
+    <mergeCell ref="B4"/>
+    <mergeCell ref="C4"/>
+    <mergeCell ref="D4"/>
+    <mergeCell ref="E4"/>
+    <mergeCell ref="F4"/>
+    <mergeCell ref="G4"/>
+    <mergeCell ref="H4"/>
+    <mergeCell ref="I4"/>
+    <mergeCell ref="J4"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>